<commit_message>
feat: shift ignore (#145)
Co-authored-by: Peter LaValle <peter.lavalle@nhs.net>
</commit_message>
<xml_diff>
--- a/tests/data/missing-id.xlsx
+++ b/tests/data/missing-id.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/peter/Documents/nuh-helper/tests/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98F310E2-AB1F-174E-84E0-D4B17C6E3C51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B06CEBF2-3F87-484A-8B96-D8C2EE37C2AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="22200" windowWidth="28800" windowHeight="15600" activeTab="1" xr2:uid="{FC40E016-DF9F-2340-ABF1-6FB1344D6D7E}"/>
+    <workbookView xWindow="9600" yWindow="22200" windowWidth="28800" windowHeight="15600" activeTab="1" xr2:uid="{FC40E016-DF9F-2340-ABF1-6FB1344D6D7E}"/>
   </bookViews>
   <sheets>
     <sheet name="description" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="33">
   <si>
     <t xml:space="preserve">version </t>
   </si>
@@ -134,6 +134,12 @@
   </si>
   <si>
     <t>oh and we skip again</t>
+  </si>
+  <si>
+    <t>nuh16</t>
+  </si>
+  <si>
+    <t>Seven</t>
   </si>
 </sst>
 </file>
@@ -549,7 +555,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9D9E2D02-7F1A-8C45-B5C7-D6826AA97033}">
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="29.83203125" customWidth="1"/>
@@ -620,6 +626,15 @@
       </c>
       <c r="C6" t="s">
         <v>19</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>31</v>
+      </c>
+      <c r="B7" s="1"/>
+      <c r="C7" t="s">
+        <v>32</v>
       </c>
     </row>
   </sheetData>

</xml_diff>